<commit_message>
Wave 2 checkpoint: technical_documents engine, plant HMB report, IEC TQ-IEC-025 revisions and review, MDL sync for new IEC tags
- technical_documents engine + doc_clause schema (clauses, parameter tables, automatic data blocks), tests
- hmb engine 1.2.0: plant heat and mass balance report (docx/pdf) with case diagrams
- IEC datasheet revisions (DS-101 B, DS-102 A, DS-103 A, DS-104 C, DS-105 A) registered and reviewed;
  DS-104 C code 2 (CPH pump data only in the TQ answer), GA comments withdrawn (EPC review error)
- 11 IEC tags added, MDL synced; lesson L-EPCE-0013

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/hmb/ALP-HMB-MAX-NG-100.xlsx
+++ b/output/hmb/ALP-HMB-MAX-NG-100.xlsx
@@ -460,7 +460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
+          <t>engine hmb v1.2.0 | data 015d1cd1c6fdda54 | 2026-09-29T03:07:46Z</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
+          <t>engine hmb v1.2.0 | data 015d1cd1c6fdda54 | 2026-09-29T03:07:46Z</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
+          <t>engine hmb v1.2.0 | data 015d1cd1c6fdda54 | 2026-09-29T03:07:46Z</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
+          <t>engine hmb v1.2.0 | data 015d1cd1c6fdda54 | 2026-09-29T03:07:46Z</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
+          <t>engine hmb v1.2.0 | data 015d1cd1c6fdda54 | 2026-09-29T03:07:46Z</t>
         </is>
       </c>
     </row>

</xml_diff>